<commit_message>
Add CSC university tier guide and ranking workbook
</commit_message>
<xml_diff>
--- a/workbooks/csc_deadlines.xlsx
+++ b/workbooks/csc_deadlines.xlsx
@@ -27,8 +27,8 @@
   <dc:title>CSC Deadlines</dc:title>
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T03:51:27Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T03:51:27Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-14T04:28:28Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-14T04:28:28Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 

</xml_diff>